<commit_message>
Refine trivia administration and preserve dashboard display preferences
</commit_message>
<xml_diff>
--- a/web/assets/trivia-question-template.xlsx
+++ b/web/assets/trivia-question-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CauHoi" sheetId="1" r:id="R1d72d30c0e5b4b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuongDan" sheetId="2" r:id="R2c70954f6fd44510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CauHoi" sheetId="1" r:id="Rd9dcdecc92ef4aaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HuongDan" sheetId="2" r:id="R10324694a3e047ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -298,11 +298,8 @@
     <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -319,18 +316,9 @@
         <x:v>Đáp án C</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>Đáp án D</x:v>
+        <x:v>Đáp án đúng</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>Đáp án E</x:v>
-      </x:c>
-      <x:c r="G1" s="4" t="str">
-        <x:v>Đáp án F</x:v>
-      </x:c>
-      <x:c r="H1" s="4" t="str">
-        <x:v>Đáp án đúng</x:v>
-      </x:c>
-      <x:c r="I1" s="4" t="str">
         <x:v>Giải thích</x:v>
       </x:c>
     </x:row>
@@ -347,13 +335,10 @@
       <x:c r="D2" s="7" t="str">
         <x:v>Không ảnh hưởng</x:v>
       </x:c>
-      <x:c r="E2" s="7" t="str"/>
-      <x:c r="F2" s="7" t="str"/>
-      <x:c r="G2" s="7" t="str"/>
-      <x:c r="H2" s="7" t="str">
+      <x:c r="E2" s="7" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="I2" s="7" t="str">
+      <x:c r="F2" s="7" t="str">
         <x:v>Hồ sơ đã và đang giải quyết quá hạn ảnh hưởng điểm tiến độ và hài lòng.</x:v>
       </x:c>
     </x:row>
@@ -364,9 +349,6 @@
       <x:c r="D3" s="7"/>
       <x:c r="E3" s="7"/>
       <x:c r="F3" s="7"/>
-      <x:c r="G3" s="7"/>
-      <x:c r="H3" s="7"/>
-      <x:c r="I3" s="7"/>
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
       <x:c r="A4" s="7"/>
@@ -375,9 +357,6 @@
       <x:c r="D4" s="7"/>
       <x:c r="E4" s="7"/>
       <x:c r="F4" s="7"/>
-      <x:c r="G4" s="7"/>
-      <x:c r="H4" s="7"/>
-      <x:c r="I4" s="7"/>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
       <x:c r="A5" s="7"/>
@@ -386,9 +365,6 @@
       <x:c r="D5" s="7"/>
       <x:c r="E5" s="7"/>
       <x:c r="F5" s="7"/>
-      <x:c r="G5" s="7"/>
-      <x:c r="H5" s="7"/>
-      <x:c r="I5" s="7"/>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="7"/>
@@ -397,9 +373,6 @@
       <x:c r="D6" s="7"/>
       <x:c r="E6" s="7"/>
       <x:c r="F6" s="7"/>
-      <x:c r="G6" s="7"/>
-      <x:c r="H6" s="7"/>
-      <x:c r="I6" s="7"/>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="7"/>
@@ -408,9 +381,6 @@
       <x:c r="D7" s="7"/>
       <x:c r="E7" s="7"/>
       <x:c r="F7" s="7"/>
-      <x:c r="G7" s="7"/>
-      <x:c r="H7" s="7"/>
-      <x:c r="I7" s="7"/>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="7"/>
@@ -419,9 +389,6 @@
       <x:c r="D8" s="7"/>
       <x:c r="E8" s="7"/>
       <x:c r="F8" s="7"/>
-      <x:c r="G8" s="7"/>
-      <x:c r="H8" s="7"/>
-      <x:c r="I8" s="7"/>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="7"/>
@@ -430,9 +397,6 @@
       <x:c r="D9" s="7"/>
       <x:c r="E9" s="7"/>
       <x:c r="F9" s="7"/>
-      <x:c r="G9" s="7"/>
-      <x:c r="H9" s="7"/>
-      <x:c r="I9" s="7"/>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="7"/>
@@ -441,9 +405,6 @@
       <x:c r="D10" s="7"/>
       <x:c r="E10" s="7"/>
       <x:c r="F10" s="7"/>
-      <x:c r="G10" s="7"/>
-      <x:c r="H10" s="7"/>
-      <x:c r="I10" s="7"/>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="7"/>
@@ -452,9 +413,6 @@
       <x:c r="D11" s="7"/>
       <x:c r="E11" s="7"/>
       <x:c r="F11" s="7"/>
-      <x:c r="G11" s="7"/>
-      <x:c r="H11" s="7"/>
-      <x:c r="I11" s="7"/>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
       <x:c r="A12" s="7"/>
@@ -463,14 +421,11 @@
       <x:c r="D12" s="7"/>
       <x:c r="E12" s="7"/>
       <x:c r="F12" s="7"/>
-      <x:c r="G12" s="7"/>
-      <x:c r="H12" s="7"/>
-      <x:c r="I12" s="7"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="H2:H501">
-      <x:formula1>"A,B,C,D,E,F"</x:formula1>
+    <x:dataValidation type="list" sqref="E2:E501">
+      <x:formula1>"A,B,C"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -516,7 +471,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Giữ nguyên tên và thứ tự 9 cột ở dòng 1. Mỗi dòng một câu hỏi.</x:v>
+        <x:v>Giữ nguyên tên và thứ tự 6 cột ở dòng 1. Mỗi dòng một câu hỏi.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="44" customHeight="1">
@@ -532,7 +487,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Có thể thêm C–F liên tục, không bỏ trống đáp án ở giữa. Mỗi đáp án tối đa 400 ký tự, không trùng nhau.</x:v>
+        <x:v>Có thể thêm đáp án C. Tối đa 3 đáp án, mỗi đáp án tối đa 400 ký tự, không trùng nhau.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
@@ -540,7 +495,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Đáp án đúng: một chữ A–F, ứng với đáp án đã nhập. Giải thích tùy chọn, tối đa 2000 ký tự.</x:v>
+        <x:v>Đáp án đúng: một chữ A–C, ứng với đáp án đã nhập. Giải thích tùy chọn, tối đa 2000 ký tự.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
@@ -564,7 +519,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Câu mới lưu Nháp. Mở từng câu để rà soát và công khai. Câu trùng nội dung câu hỏi được bỏ qua, không sửa câu đã có.</x:v>
+        <x:v>Câu mới lưu Nháp. Bấm Duyệt công khai sau khi rà soát. Câu trùng được bỏ qua. File mẫu cũ phải để trống D, E, F.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>